<commit_message>
Refactor: Vite + modularización + nuevas funcionalidades
- Migrado a Vite como bundler
- Código modularizado en src/ (9 módulos ES6)
- Toast notifications reemplazan alert()
- Sonido al escanear (Web Audio API)
- Skeleton loading + paginación en tabla
- Historial de escaneos (colección scans)
- Botón Vender con registro en ventas
- Exportar productos a Excel
- Generación multi-formato (EAN8/13, UPC, CODE128, etc.)
- Subida de imágenes a Firebase Storage
- Escaneo batch con export CSV
- Soft delete (active: false)
- Dashboard con Chart.js (stats, charts, ventas)
- Service Worker para modo offline
- Tests unitarios con Vitest
</commit_message>
<xml_diff>
--- a/stock/Stock.xlsx
+++ b/stock/Stock.xlsx
@@ -10267,12 +10267,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -10289,7 +10295,7 @@
       <alignment vertical="top"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -10304,6 +10310,15 @@
     </xf>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -46844,29 +46859,29 @@
         <v>472</v>
       </c>
     </row>
-    <row r="1395" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1395" s="3" t="s">
+    <row r="1395" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1395" s="5" t="s">
         <v>2494</v>
       </c>
-      <c r="B1395" s="3" t="s">
+      <c r="B1395" s="5" t="s">
         <v>3230</v>
       </c>
-      <c r="C1395" s="3" t="s">
+      <c r="C1395" s="5" t="s">
         <v>511</v>
       </c>
-      <c r="D1395" s="3" t="s">
+      <c r="D1395" s="5" t="s">
         <v>597</v>
       </c>
-      <c r="E1395" s="4">
+      <c r="E1395" s="6">
         <v>2</v>
       </c>
-      <c r="F1395" s="4">
+      <c r="F1395" s="6">
         <v>59000</v>
       </c>
-      <c r="G1395" s="4">
+      <c r="G1395" s="6">
         <v>30599.09</v>
       </c>
-      <c r="H1395" s="3" t="s">
+      <c r="H1395" s="5" t="s">
         <v>472</v>
       </c>
     </row>
@@ -51742,29 +51757,29 @@
         <v>3406</v>
       </c>
     </row>
-    <row r="1604" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1604" s="3" t="s">
+    <row r="1604" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1604" s="5" t="s">
         <v>2779</v>
       </c>
-      <c r="B1604" s="3" t="s">
+      <c r="B1604" s="5" t="s">
         <v>2780</v>
       </c>
-      <c r="C1604" s="3" t="s">
+      <c r="C1604" s="5" t="s">
         <v>572</v>
       </c>
-      <c r="D1604" s="3" t="s">
+      <c r="D1604" s="5" t="s">
         <v>572</v>
       </c>
-      <c r="E1604" s="4">
-        <v>1</v>
-      </c>
-      <c r="F1604" s="4">
+      <c r="E1604" s="6">
+        <v>1</v>
+      </c>
+      <c r="F1604" s="6">
         <v>4500</v>
       </c>
-      <c r="G1604" s="4">
+      <c r="G1604" s="6">
         <v>7721.96</v>
       </c>
-      <c r="H1604" s="3" t="s">
+      <c r="H1604" s="5" t="s">
         <v>3390</v>
       </c>
     </row>

</xml_diff>